<commit_message>
cadastrar nova microrrede MG2
</commit_message>
<xml_diff>
--- a/exemplos/DADOS MR 2.xlsx
+++ b/exemplos/DADOS MR 2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/11a919a0b67208fd/Área de Trabalho/01 - DOCUMENTOS/claudia/claudia_tese v2/exemplos/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a7044ff72ef9da91/Desktop/Doutorado/2026/Caracterização das cargas das MRs por estação/MRs para inserir no algoritimo/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{4A94543C-C25B-467A-A115-E8E5E51082D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="26" documentId="8_{6AC3D7AE-85C3-40ED-9177-F6A4F5AFD2DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4E7A0013-5D60-4744-BDDF-157DE9F09082}"/>
   <bookViews>
-    <workbookView xWindow="28692" yWindow="-108" windowWidth="29016" windowHeight="15696" activeTab="3" xr2:uid="{65A26838-979D-467E-8ADD-70D8D5EE1CD9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{65A26838-979D-467E-8ADD-70D8D5EE1CD9}"/>
   </bookViews>
   <sheets>
     <sheet name="MR 2 - VERÃO" sheetId="1" r:id="rId1"/>
@@ -18,28 +18,17 @@
     <sheet name="MR 2 - INVERNO" sheetId="3" r:id="rId3"/>
     <sheet name="MR 2 - PRIMAVERA" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="46">
   <si>
     <t>Descrição da Carga</t>
   </si>
@@ -111,15 +100,6 @@
   </si>
   <si>
     <t>Tanque L</t>
-  </si>
-  <si>
-    <t>Consumo (L/kWh) 100%</t>
-  </si>
-  <si>
-    <t>Consumo (L/kWh) 75%</t>
-  </si>
-  <si>
-    <t>Consumo (L/kWh) 50%</t>
   </si>
   <si>
     <t>Cap de descarga (kWh)</t>
@@ -255,9 +235,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office 2013 - 2022">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -295,7 +275,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -401,7 +381,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -543,7 +523,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -552,24 +532,24 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9676991-DE06-438B-B13F-309B9837D3E6}">
   <dimension ref="A1:K44"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.88671875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="22.44140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="21.44140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="21.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -589,7 +569,7 @@
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
@@ -608,7 +588,7 @@
       <c r="I3" s="2"/>
       <c r="J3" s="2"/>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>6</v>
       </c>
@@ -627,7 +607,7 @@
       <c r="I4" s="2"/>
       <c r="J4" s="2"/>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>7</v>
       </c>
@@ -646,7 +626,7 @@
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>8</v>
       </c>
@@ -665,7 +645,7 @@
       <c r="I6" s="2"/>
       <c r="J6" s="2"/>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>9</v>
       </c>
@@ -684,7 +664,7 @@
       <c r="I7" s="2"/>
       <c r="J7" s="2"/>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>10</v>
       </c>
@@ -703,7 +683,7 @@
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>8</v>
       </c>
@@ -720,9 +700,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B10" s="2">
         <v>66.599999999999994</v>
@@ -737,9 +717,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B11" s="2">
         <v>88.8</v>
@@ -754,9 +734,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B12" s="2">
         <v>0.01</v>
@@ -771,9 +751,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B13" s="2">
         <v>1</v>
@@ -788,9 +768,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="B14" s="2">
         <v>1</v>
@@ -805,9 +785,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B15" s="2">
         <v>1</v>
@@ -822,7 +802,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>11</v>
       </c>
@@ -839,7 +819,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>12</v>
       </c>
@@ -856,7 +836,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>13</v>
       </c>
@@ -873,7 +853,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>14</v>
       </c>
@@ -890,7 +870,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>15</v>
       </c>
@@ -907,7 +887,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>16</v>
       </c>
@@ -924,7 +904,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>17</v>
       </c>
@@ -941,7 +921,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>18</v>
       </c>
@@ -958,21 +938,21 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="2"/>
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
       <c r="D24" s="2"/>
       <c r="E24" s="2"/>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="2"/>
       <c r="B25" s="2"/>
       <c r="C25" s="2"/>
       <c r="D25" s="2"/>
       <c r="E25" s="2"/>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>19</v>
       </c>
@@ -989,27 +969,27 @@
         <v>23</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="H26" s="1" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="I26" s="1" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="J26" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B27" s="2">
-        <v>160</v>
+        <v>175</v>
       </c>
       <c r="C27" s="2">
         <v>0.2</v>
@@ -1022,9 +1002,9 @@
       <c r="I27" s="2"/>
       <c r="J27" s="2"/>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B28" s="2">
         <v>13</v>
@@ -1050,12 +1030,12 @@
       <c r="I28" s="2"/>
       <c r="J28" s="2"/>
       <c r="K28" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B29" s="2">
         <v>33</v>
@@ -1074,15 +1054,15 @@
         <v>175</v>
       </c>
       <c r="J29" s="2" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="K29" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="B30" s="2"/>
       <c r="C30" s="2">
@@ -1096,109 +1076,83 @@
       <c r="I30" s="2"/>
       <c r="J30" s="2"/>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" s="2"/>
       <c r="B31" s="2"/>
       <c r="C31" s="2"/>
       <c r="D31" s="2"/>
       <c r="E31" s="2"/>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" s="2"/>
       <c r="B32" s="2"/>
       <c r="C32" s="2"/>
       <c r="D32" s="2"/>
       <c r="E32" s="2"/>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" s="2"/>
       <c r="B33" s="2"/>
       <c r="C33" s="2"/>
       <c r="D33" s="2"/>
       <c r="E33" s="2"/>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
       <c r="D34" s="2"/>
       <c r="E34" s="2"/>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" s="2"/>
       <c r="B35" s="2"/>
       <c r="C35" s="2"/>
       <c r="D35" s="2"/>
       <c r="E35" s="2"/>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" s="2"/>
       <c r="B36" s="2"/>
       <c r="C36" s="2"/>
       <c r="D36" s="2"/>
       <c r="E36" s="2"/>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" s="2"/>
       <c r="B37" s="2"/>
       <c r="C37" s="2"/>
       <c r="D37" s="2"/>
       <c r="E37" s="2"/>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" s="2"/>
       <c r="B38" s="2"/>
       <c r="C38" s="2"/>
       <c r="D38" s="2"/>
       <c r="E38" s="2"/>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C39" s="2"/>
       <c r="D39" s="2"/>
       <c r="E39" s="2"/>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A40" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="B40" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="C40" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D40" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="E40" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="F40" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="G40" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="H40" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="I40" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="J40" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A41" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="B41" s="2">
-        <v>100</v>
-      </c>
-      <c r="C41" s="2">
-        <v>0.3</v>
-      </c>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A40" s="1"/>
+      <c r="B40" s="1"/>
+      <c r="C40" s="1"/>
+      <c r="D40" s="1"/>
+      <c r="E40" s="1"/>
+      <c r="F40" s="1"/>
+      <c r="G40" s="1"/>
+      <c r="H40" s="1"/>
+      <c r="I40" s="1"/>
+      <c r="J40" s="1"/>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A41" s="2"/>
+      <c r="B41" s="2"/>
+      <c r="C41" s="2"/>
       <c r="D41" s="2"/>
       <c r="E41" s="2"/>
       <c r="F41" s="2"/>
@@ -1207,67 +1161,34 @@
       <c r="I41" s="2"/>
       <c r="J41" s="2"/>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A42" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="B42" s="2">
-        <v>5.5</v>
-      </c>
-      <c r="C42" s="2">
-        <v>2</v>
-      </c>
-      <c r="D42" s="2">
-        <v>24</v>
-      </c>
-      <c r="E42" s="2">
-        <v>40</v>
-      </c>
-      <c r="F42" s="2">
-        <v>0.3</v>
-      </c>
-      <c r="G42" s="2">
-        <v>0.35</v>
-      </c>
-      <c r="H42" s="2">
-        <v>0.4</v>
-      </c>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A42" s="2"/>
+      <c r="B42" s="2"/>
+      <c r="C42" s="2"/>
+      <c r="D42" s="2"/>
+      <c r="E42" s="2"/>
+      <c r="F42" s="2"/>
+      <c r="G42" s="2"/>
+      <c r="H42" s="2"/>
       <c r="I42" s="2"/>
       <c r="J42" s="2"/>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A43" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="B43" s="2">
-        <v>30</v>
-      </c>
-      <c r="C43" s="2">
-        <v>0.8</v>
-      </c>
-      <c r="D43" s="2">
-        <v>4</v>
-      </c>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A43" s="2"/>
+      <c r="B43" s="2"/>
+      <c r="C43" s="2"/>
+      <c r="D43" s="2"/>
       <c r="E43" s="2"/>
       <c r="F43" s="2"/>
       <c r="G43" s="2"/>
       <c r="H43" s="2"/>
-      <c r="I43" s="2">
-        <f>150*60</f>
-        <v>9000</v>
-      </c>
-      <c r="J43" s="2" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A44" s="2" t="s">
-        <v>33</v>
-      </c>
+      <c r="I43" s="2"/>
+      <c r="J43" s="2"/>
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A44" s="2"/>
       <c r="B44" s="2"/>
-      <c r="C44" s="2">
-        <v>0.87</v>
-      </c>
+      <c r="C44" s="2"/>
       <c r="D44" s="2"/>
       <c r="E44" s="2"/>
       <c r="F44" s="2"/>
@@ -1284,25 +1205,25 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{906671BA-8876-4FEB-AD5C-EE1D43EC6D92}">
   <dimension ref="A1:K30"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.88671875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="22.44140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="21.44140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="21.5546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="7.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1322,7 +1243,7 @@
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
@@ -1341,7 +1262,7 @@
       <c r="I3" s="2"/>
       <c r="J3" s="2"/>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>6</v>
       </c>
@@ -1360,7 +1281,7 @@
       <c r="I4" s="2"/>
       <c r="J4" s="2"/>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>7</v>
       </c>
@@ -1379,7 +1300,7 @@
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>8</v>
       </c>
@@ -1398,7 +1319,7 @@
       <c r="I6" s="2"/>
       <c r="J6" s="2"/>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>9</v>
       </c>
@@ -1417,7 +1338,7 @@
       <c r="I7" s="2"/>
       <c r="J7" s="2"/>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>10</v>
       </c>
@@ -1436,7 +1357,7 @@
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>8</v>
       </c>
@@ -1453,9 +1374,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B10" s="2">
         <v>12.1</v>
@@ -1470,9 +1391,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B11" s="2">
         <v>16</v>
@@ -1487,9 +1408,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B12" s="2">
         <v>0.01</v>
@@ -1504,9 +1425,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B13" s="2">
         <v>1</v>
@@ -1521,9 +1442,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="B14" s="2">
         <v>1</v>
@@ -1538,9 +1459,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B15" s="2">
         <v>1</v>
@@ -1555,7 +1476,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>11</v>
       </c>
@@ -1572,7 +1493,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>12</v>
       </c>
@@ -1589,7 +1510,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>13</v>
       </c>
@@ -1606,7 +1527,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>14</v>
       </c>
@@ -1623,7 +1544,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>15</v>
       </c>
@@ -1640,7 +1561,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>16</v>
       </c>
@@ -1657,7 +1578,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>17</v>
       </c>
@@ -1674,7 +1595,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>18</v>
       </c>
@@ -1691,21 +1612,21 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="2"/>
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
       <c r="D24" s="2"/>
       <c r="E24" s="2"/>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="2"/>
       <c r="B25" s="2"/>
       <c r="C25" s="2"/>
       <c r="D25" s="2"/>
       <c r="E25" s="2"/>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>19</v>
       </c>
@@ -1722,27 +1643,27 @@
         <v>23</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="H26" s="1" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="I26" s="1" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="J26" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B27" s="2">
-        <v>160</v>
+        <v>175</v>
       </c>
       <c r="C27" s="2">
         <v>0.2</v>
@@ -1755,9 +1676,9 @@
       <c r="I27" s="2"/>
       <c r="J27" s="2"/>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B28" s="2">
         <v>13</v>
@@ -1783,12 +1704,12 @@
       <c r="I28" s="2"/>
       <c r="J28" s="2"/>
       <c r="K28" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B29" s="2">
         <v>33</v>
@@ -1804,19 +1725,18 @@
       <c r="G29" s="2"/>
       <c r="H29" s="2"/>
       <c r="I29" s="2">
-        <f>150*60</f>
-        <v>9000</v>
+        <v>175</v>
       </c>
       <c r="J29" s="2" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="K29" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="B30" s="2"/>
       <c r="C30" s="2">
@@ -1838,24 +1758,24 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5359127-CCC8-40E8-82BF-9F5FFA21648E}">
   <dimension ref="A1:K30"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.88671875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="22.44140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="21.44140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="21.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1875,7 +1795,7 @@
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
@@ -1894,7 +1814,7 @@
       <c r="I3" s="2"/>
       <c r="J3" s="2"/>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>6</v>
       </c>
@@ -1913,7 +1833,7 @@
       <c r="I4" s="2"/>
       <c r="J4" s="2"/>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>7</v>
       </c>
@@ -1932,7 +1852,7 @@
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>8</v>
       </c>
@@ -1951,7 +1871,7 @@
       <c r="I6" s="2"/>
       <c r="J6" s="2"/>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>9</v>
       </c>
@@ -1970,7 +1890,7 @@
       <c r="I7" s="2"/>
       <c r="J7" s="2"/>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>10</v>
       </c>
@@ -1989,7 +1909,7 @@
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>8</v>
       </c>
@@ -2006,9 +1926,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B10" s="2">
         <v>0</v>
@@ -2023,9 +1943,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B11" s="2">
         <v>0</v>
@@ -2040,9 +1960,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B12" s="2">
         <v>0.01</v>
@@ -2057,9 +1977,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B13" s="2">
         <v>1</v>
@@ -2074,9 +1994,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="B14" s="2">
         <v>1</v>
@@ -2091,9 +2011,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B15" s="2">
         <v>1</v>
@@ -2108,7 +2028,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>11</v>
       </c>
@@ -2125,7 +2045,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>12</v>
       </c>
@@ -2142,7 +2062,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>13</v>
       </c>
@@ -2159,7 +2079,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>14</v>
       </c>
@@ -2176,7 +2096,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>15</v>
       </c>
@@ -2193,7 +2113,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>16</v>
       </c>
@@ -2210,7 +2130,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>17</v>
       </c>
@@ -2227,7 +2147,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>18</v>
       </c>
@@ -2244,21 +2164,21 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="2"/>
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
       <c r="D24" s="2"/>
       <c r="E24" s="2"/>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="2"/>
       <c r="B25" s="2"/>
       <c r="C25" s="2"/>
       <c r="D25" s="2"/>
       <c r="E25" s="2"/>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>19</v>
       </c>
@@ -2275,27 +2195,27 @@
         <v>23</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="H26" s="1" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="I26" s="1" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="J26" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B27" s="2">
-        <v>160</v>
+        <v>175</v>
       </c>
       <c r="C27" s="2">
         <v>0.2</v>
@@ -2308,9 +2228,9 @@
       <c r="I27" s="2"/>
       <c r="J27" s="2"/>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B28" s="2">
         <v>13</v>
@@ -2336,12 +2256,12 @@
       <c r="I28" s="2"/>
       <c r="J28" s="2"/>
       <c r="K28" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B29" s="2">
         <v>33</v>
@@ -2357,19 +2277,18 @@
       <c r="G29" s="2"/>
       <c r="H29" s="2"/>
       <c r="I29" s="2">
-        <f>150*60</f>
-        <v>9000</v>
+        <v>175</v>
       </c>
       <c r="J29" s="2" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="K29" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="B30" s="2"/>
       <c r="C30" s="2">
@@ -2391,24 +2310,24 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5810F99-7DD3-4AE0-A0D7-12D8107F717C}">
   <dimension ref="A1:K30"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.88671875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="22.44140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="21.44140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="21.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -2428,7 +2347,7 @@
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
@@ -2447,7 +2366,7 @@
       <c r="I3" s="2"/>
       <c r="J3" s="2"/>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>6</v>
       </c>
@@ -2466,7 +2385,7 @@
       <c r="I4" s="2"/>
       <c r="J4" s="2"/>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>7</v>
       </c>
@@ -2485,7 +2404,7 @@
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>8</v>
       </c>
@@ -2504,7 +2423,7 @@
       <c r="I6" s="2"/>
       <c r="J6" s="2"/>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>9</v>
       </c>
@@ -2523,7 +2442,7 @@
       <c r="I7" s="2"/>
       <c r="J7" s="2"/>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>10</v>
       </c>
@@ -2542,7 +2461,7 @@
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>8</v>
       </c>
@@ -2559,9 +2478,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B10" s="2">
         <v>54.5</v>
@@ -2576,9 +2495,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B11" s="2">
         <v>72</v>
@@ -2593,9 +2512,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B12" s="2">
         <v>0.01</v>
@@ -2610,9 +2529,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B13" s="2">
         <v>1</v>
@@ -2627,9 +2546,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="B14" s="2">
         <v>1</v>
@@ -2644,9 +2563,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B15" s="2">
         <v>1</v>
@@ -2661,7 +2580,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>11</v>
       </c>
@@ -2678,7 +2597,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>12</v>
       </c>
@@ -2695,7 +2614,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>13</v>
       </c>
@@ -2712,7 +2631,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>14</v>
       </c>
@@ -2729,7 +2648,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>15</v>
       </c>
@@ -2746,7 +2665,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>16</v>
       </c>
@@ -2763,7 +2682,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>17</v>
       </c>
@@ -2780,7 +2699,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>18</v>
       </c>
@@ -2797,21 +2716,21 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="2"/>
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
       <c r="D24" s="2"/>
       <c r="E24" s="2"/>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="2"/>
       <c r="B25" s="2"/>
       <c r="C25" s="2"/>
       <c r="D25" s="2"/>
       <c r="E25" s="2"/>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>19</v>
       </c>
@@ -2828,27 +2747,27 @@
         <v>23</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="H26" s="1" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="I26" s="1" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="J26" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B27" s="2">
-        <v>160</v>
+        <v>175</v>
       </c>
       <c r="C27" s="2">
         <v>0.2</v>
@@ -2861,9 +2780,9 @@
       <c r="I27" s="2"/>
       <c r="J27" s="2"/>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B28" s="2">
         <v>13</v>
@@ -2889,12 +2808,12 @@
       <c r="I28" s="2"/>
       <c r="J28" s="2"/>
       <c r="K28" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B29" s="2">
         <v>33</v>
@@ -2910,19 +2829,18 @@
       <c r="G29" s="2"/>
       <c r="H29" s="2"/>
       <c r="I29" s="2">
-        <f>150*60</f>
-        <v>9000</v>
+        <v>175</v>
       </c>
       <c r="J29" s="2" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="K29" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="B30" s="2"/>
       <c r="C30" s="2">

</xml_diff>

<commit_message>
add tempo de execução
</commit_message>
<xml_diff>
--- a/exemplos/DADOS MR 2.xlsx
+++ b/exemplos/DADOS MR 2.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="49">
   <si>
     <t>MR 2 - VERÃO</t>
   </si>
@@ -130,6 +130,9 @@
     <t>PV</t>
   </si>
   <si>
+    <t>200</t>
+  </si>
+  <si>
     <t>Diesel</t>
   </si>
   <si>
@@ -137,6 +140,9 @@
   </si>
   <si>
     <t>Bateria</t>
+  </si>
+  <si>
+    <t>40</t>
   </si>
   <si>
     <t>10500</t>
@@ -980,8 +986,8 @@
       <c r="A27" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B27" s="2">
-        <v>175</v>
+      <c r="B27" s="2" t="s">
+        <v>37</v>
       </c>
       <c r="C27" s="2">
         <v>0.2</v>
@@ -996,7 +1002,7 @@
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B28" s="2">
         <v>13</v>
@@ -1022,15 +1028,15 @@
       <c r="I28" s="2"/>
       <c r="J28" s="2"/>
       <c r="K28" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="B29" s="2">
-        <v>33</v>
+        <v>40</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>41</v>
       </c>
       <c r="C29" s="2">
         <v>0.7</v>
@@ -1043,18 +1049,18 @@
       <c r="G29" s="2"/>
       <c r="H29" s="2"/>
       <c r="I29" s="2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="J29" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="K29" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B30" s="2"/>
       <c r="C30" s="2">
@@ -1212,7 +1218,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
@@ -1654,8 +1660,8 @@
       <c r="A27" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B27" s="2">
-        <v>175</v>
+      <c r="B27" s="2" t="s">
+        <v>37</v>
       </c>
       <c r="C27" s="2">
         <v>0.2</v>
@@ -1670,7 +1676,7 @@
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B28" s="2">
         <v>13</v>
@@ -1696,15 +1702,15 @@
       <c r="I28" s="2"/>
       <c r="J28" s="2"/>
       <c r="K28" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="B29" s="2">
-        <v>33</v>
+        <v>40</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>41</v>
       </c>
       <c r="C29" s="2">
         <v>0.7</v>
@@ -1717,18 +1723,18 @@
       <c r="G29" s="2"/>
       <c r="H29" s="2"/>
       <c r="I29" s="2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="J29" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="K29" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B30" s="2"/>
       <c r="C30" s="2">
@@ -1764,7 +1770,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
@@ -2206,8 +2212,8 @@
       <c r="A27" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B27" s="2">
-        <v>175</v>
+      <c r="B27" s="2" t="s">
+        <v>37</v>
       </c>
       <c r="C27" s="2">
         <v>0.2</v>
@@ -2222,7 +2228,7 @@
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B28" s="2">
         <v>13</v>
@@ -2248,15 +2254,15 @@
       <c r="I28" s="2"/>
       <c r="J28" s="2"/>
       <c r="K28" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="B29" s="2">
-        <v>33</v>
+        <v>40</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>41</v>
       </c>
       <c r="C29" s="2">
         <v>0.7</v>
@@ -2269,18 +2275,18 @@
       <c r="G29" s="2"/>
       <c r="H29" s="2"/>
       <c r="I29" s="2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="J29" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="K29" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B30" s="2"/>
       <c r="C30" s="2">
@@ -2316,7 +2322,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
@@ -2758,8 +2764,8 @@
       <c r="A27" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B27" s="2">
-        <v>175</v>
+      <c r="B27" s="2" t="s">
+        <v>37</v>
       </c>
       <c r="C27" s="2">
         <v>0.2</v>
@@ -2774,7 +2780,7 @@
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B28" s="2">
         <v>13</v>
@@ -2800,15 +2806,15 @@
       <c r="I28" s="2"/>
       <c r="J28" s="2"/>
       <c r="K28" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="B29" s="2">
-        <v>33</v>
+        <v>40</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>41</v>
       </c>
       <c r="C29" s="2">
         <v>0.7</v>
@@ -2821,18 +2827,18 @@
       <c r="G29" s="2"/>
       <c r="H29" s="2"/>
       <c r="I29" s="2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="J29" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="K29" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B30" s="2"/>
       <c r="C30" s="2">

</xml_diff>